<commit_message>
feat: Enhance weather data fetching and error handling
- Improved .env file loading with error raising if it fails.
- Added threading support in WeatherScheduler for parallel weather data fetching.
- Updated WeatherAPI to include timeout parameter and better error logging.
- Cleaned up logging messages for clarity and consistency.
- Ensured city data is valid before appending to Excel.
</commit_message>
<xml_diff>
--- a/cities.xlsx
+++ b/cities.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dev\Vs Code Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B88C7E73-E114-4936-9160-15C97C5BF6CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3AFCFFF-B640-407E-9179-031103BA1787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>City</t>
   </si>
@@ -37,6 +37,15 @@
   </si>
   <si>
     <t>Karachi</t>
+  </si>
+  <si>
+    <t>Quetta</t>
+  </si>
+  <si>
+    <t>Peshawar</t>
+  </si>
+  <si>
+    <t>Lahore</t>
   </si>
 </sst>
 </file>
@@ -354,7 +363,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -377,6 +386,21 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>